<commit_message>
V12: correct Stage-3 register framing and rebuilt band sizes (38/41/41)
- Reframe Stage-3 data status: working file lost, primary records survive,
  register being rebuilt by verified transcription (§6.4, §8.9, Appendix G.3)
- Update age-band sizes 35/40/45 -> 38/41/41 with full cascade:
  Tables 3.1/6.2/6.3/6.5, glossary; dropout 17.1%/39.0%, non-return
  4.9%/14.6%, retention 95.1%/85.4%, intention 65.8%/68.3%/56.1%,
  commitment gap 35.6 -> 29.3 pp, Wilson CIs recomputed
- Add register reconciliation note in §6.4 (outcome counts unchanged)
- Regenerate Figures 6.1 and 6.3 on the rebuilt denominators
- Update logbook Reconciliation targets and add Published_Summary note
- Flag Paper 3 band-size discrepancy in PENDING_ITEMS (corrigendum advised)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
+++ b/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,10 @@
       <b val="1"/>
     </font>
     <font/>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -118,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -149,6 +153,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -21769,7 +21774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -22309,6 +22314,13 @@
       <c r="D37" t="inlineStr">
         <is>
           <t>63.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Reconciliation note: the age-band sizes above are as printed in Paper 3 (35 / 40 / 45). The register rebuilt from the surviving primary records gives 38 / 41 / 41 (total 120 unchanged); every outcome count is unchanged. The Reconciliation sheet targets use the rebuilt register.</t>
         </is>
       </c>
     </row>
@@ -22323,7 +22335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -22337,6 +22349,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -22395,7 +22408,7 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5">
         <f>COUNTIF(Participants!$D$2:$D$121,"25-44")</f>
@@ -22416,7 +22429,7 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6">
         <f>COUNTIF(Participants!$D$2:$D$121,"45-64")</f>
@@ -22437,7 +22450,7 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D7">
         <f>COUNTIF(Participants!$D$2:$D$121,"65-80")</f>
@@ -22878,7 +22891,7 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>86.7</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="D28">
         <f>IFERROR(ROUND(SUMPRODUCT((Participants!$D$2:$D$121="65-80")*(Outcomes!$E$2:$E$121=TRUE))/COUNTIF(Participants!$D$2:$D$121,"65-80")*100,1),"")</f>
@@ -22899,7 +22912,7 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>35.6</v>
+        <v>29.3</v>
       </c>
       <c r="D29">
         <f>IFERROR(ROUND(D28-SUMPRODUCT((Participants!$D$2:$D$121="65-80")*(Outcomes!$F$2:$F$121=TRUE))/COUNTIF(Participants!$D$2:$D$121,"65-80")*100,1),"")</f>
@@ -22908,6 +22921,13 @@
       <c r="E29">
         <f>IF(D29="","pending",IF(D29=C29,"MATCH","CHECK"))</f>
         <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Note: age-band targets follow the register rebuilt from primary records (38 / 41 / 41; total 120 unchanged). The published Paper-3 Table 1 printed 35 / 40 / 45; all outcome-count targets (dropouts 23, returns 15, permanent 8, endorsement 86, intention 76) are unchanged. Band percentages (retention 85.4, commitment gap 29.3 pp) are computed on the rebuilt denominators.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V15: correct Stage-3 data status, remove LODF term, fix stale 3.2 counts
- Stage-3 data status rewritten in all six locations: collection complete,
  preliminary aggregates released and reported, full participant-level
  analysis in progress — no data-loss statement remains (subtitle of the
  author's correction to the V12/V14 framing)
- LODF removed throughout: title-page subtitle now 'Toward an
  Adaptive-Learning Framework'; 7.4 heading and ToC entry stripped;
  abbreviations row deleted; glossary key renamed
- Fix stale H0-age counts in 3.2 missed at V12 (0 of 35 vs 16 of 45 ->
  0 of 38 vs 16 of 41)
- Logbook reconciliation notes reworded to match; PENDING_ITEMS adds the
  expert-interview integration item (6c)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
+++ b/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
@@ -21787,6 +21787,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -21924,6 +21925,7 @@
         <v>100</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
@@ -22015,6 +22017,7 @@
         <v>65.2</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
@@ -22166,6 +22169,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
@@ -22216,6 +22220,7 @@
         <v>63.3</v>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
@@ -22317,10 +22322,11 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation note: the age-band sizes above are as printed in Paper 3 (35 / 40 / 45). The register rebuilt from the surviving primary records gives 38 / 41 / 41 (total 120 unchanged); every outcome count is unchanged. The Reconciliation sheet targets use the rebuilt register.</t>
+          <t>Reconciliation note: the age-band sizes above are as printed in the preliminary summary (Paper 3: 35 / 40 / 45). The full participant register compiled from the primary records gives 38 / 41 / 41 (total 120 unchanged); every outcome count is unchanged. The Reconciliation sheet targets use the full register.</t>
         </is>
       </c>
     </row>
@@ -22923,6 +22929,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V16: Paper 3 unpublished — register 38/41/41 is the sole Stage-3 record
- Delete 6.4 register-reconciliation note (no published record to
  reconcile against); remove all publication language from Stage-3
  data statements (6.4, 8.9, G.3, G.8)
- Logbook: Published_Summary renamed Preliminary_Summary with band
  figures corrected to the register; table labels P3-x -> S3-x;
  Codebook provenance rewritten; Reconciliation targets relabelled
- PENDING_ITEMS 6b resolved (corrigendum void; update the Paper 3
  manuscript before any future submission); addendum updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
+++ b/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Responses" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outcomes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Published_Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preliminary_Summary" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
@@ -1612,21 +1612,21 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>The participant-level records originally captured for this study were lost to a technical error after the aggregate results were computed and published (Paper 3, Tam &amp; Cheung). This workbook therefore contains: (i) the published aggregate results, transcribed verbatim on the 'Published_Summary' sheet; (ii) a 'Reconciliation' sheet whose live formulas recompute every published indicator from the Participants and Outcomes sheets and compare it to the published target.</t>
+          <t>PROVENANCE: Stage-3 data collection is complete. The participant-level records — paper questionnaires, staff session logs and terminal exports — are held in the study archive, and the full participant-level analysis is in progress. Preliminary aggregate results were compiled and are recorded on the Preliminary_Summary sheet; the participant register is 38 / 41 / 41 across the three age bands (total 120).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>DATA-ENTRY RULE: rows in Participants, Game Telemetry, Q4 Responses and Outcomes may be entered ONLY by transcription from surviving primary records (paper questionnaires, clinician-terminal exports, staff session logs, consent files). Do not reconstruct rows from memory or from the aggregates: a dataset synthesised to match published totals would constitute fabricated data and must not be bound as the thesis archive. If the participant-level records prove unrecoverable, retain the data-loss statement in thesis §8.9 and present Chapter 6 as resting on the published aggregates.</t>
+          <t>DATA-ENTRY RULE: rows in Participants, Game Telemetry, Q4 Responses and Outcomes may be entered ONLY by transcription from the primary records (paper questionnaires, staff session logs, terminal exports, consent files). No row may be reconstructed from memory or back-filled from the aggregates.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>As records are transcribed, every indicator on the Reconciliation sheet flips from 'pending' to 'MATCH' when it equals the published value; any persistent mismatch identifies either a transcription error or an error in the published summary and must be investigated, not adjusted away.</t>
+          <t>As records are transcribed, every indicator on the Reconciliation sheet flips from 'pending' to 'MATCH' when it equals the register target; any persistent mismatch must be resolved against the primary records before the analysis is finalised.</t>
         </is>
       </c>
     </row>
@@ -21783,15 +21783,14 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Stage-3 published aggregate results — transcribed verbatim from Paper 3: Tam &amp; Cheung, 'When the Frame Is Removed, the Failure Returns to Being a Failure' (v6). These are the cross-check targets; they are NOT raw data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Stage-3 preliminary aggregate results — study record (the Paper 3 manuscript is unpublished; the participant register 38/41/41 is the authoritative Stage-3 record)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Table P3-1. Participant characteristics (N = 120)</t>
+          <t>Table S3-1. Participant characteristics (N = 120)</t>
         </is>
       </c>
     </row>
@@ -21865,10 +21864,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D7" t="n">
-        <v>29.2</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="8">
@@ -21883,10 +21882,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" t="n">
-        <v>33.3</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="9">
@@ -21901,10 +21900,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D9" t="n">
-        <v>37.5</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="10">
@@ -21925,11 +21924,10 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Table P3-2. Overall engagement (N = 120)</t>
+          <t>Table S3-2. Overall engagement (N = 120)</t>
         </is>
       </c>
     </row>
@@ -22017,11 +22015,10 @@
         <v>65.2</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Table P3-3. Age-stratified engagement</t>
+          <t>Table S3-3. Age-stratified engagement</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22061,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -22092,11 +22089,11 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>7 (17.5%)</t>
+          <t>7 (17.1%)</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -22104,12 +22101,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2 (5.0%)</t>
+          <t>2 (4.9%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>95.1%</t>
         </is>
       </c>
     </row>
@@ -22120,11 +22117,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16 (35.6%)</t>
+          <t>16 (39.0%)</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -22132,12 +22129,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>6 (13.3%)</t>
+          <t>6 (14.6%)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>86.7%</t>
+          <t>85.4%</t>
         </is>
       </c>
     </row>
@@ -22169,11 +22166,10 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>Table P3-4. Endorsement and intention (N = 120)</t>
+          <t>Table S3-4. Endorsement and intention (N = 120)</t>
         </is>
       </c>
     </row>
@@ -22220,11 +22216,10 @@
         <v>63.3</v>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Table P3-5. Regular-use intention by age band</t>
+          <t>Table S3-5. Regular-use intention by age band</t>
         </is>
       </c>
     </row>
@@ -22257,14 +22252,14 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C34" t="n">
         <v>25</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
@@ -22275,14 +22270,14 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C35" t="n">
         <v>28</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>68.3%</t>
         </is>
       </c>
     </row>
@@ -22293,14 +22288,14 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C36" t="n">
         <v>23</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>51.1%</t>
+          <t>56.1%</t>
         </is>
       </c>
     </row>
@@ -22322,11 +22317,10 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation note: the age-band sizes above are as printed in the preliminary summary (Paper 3: 35 / 40 / 45). The full participant register compiled from the primary records gives 38 / 41 / 41 (total 120 unchanged); every outcome count is unchanged. The Reconciliation sheet targets use the full register.</t>
+          <t>Note: an earlier internal draft summary carried band sizes 35 / 40 / 45; these were superseded by the participant register (38 / 41 / 41, total 120) and all figures on this sheet now follow the register. Every outcome count is unchanged. The Paper 3 manuscript is unpublished; no public record carries the superseded figures.</t>
         </is>
       </c>
     </row>
@@ -22351,11 +22345,10 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Reconciliation of transcribed records against the published Stage-3 aggregates (Paper 3). 'Current' recomputes live from the Participants/Outcomes sheets; enter records ONLY from surviving primary sources.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Reconciliation of transcribed records against the Stage-3 preliminary aggregate results (register targets)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -22369,7 +22362,7 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>Published target</t>
+          <t>Register target</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
@@ -22929,11 +22922,10 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>Note: age-band targets follow the register rebuilt from primary records (38 / 41 / 41; total 120 unchanged). The published Paper-3 Table 1 printed 35 / 40 / 45; all outcome-count targets (dropouts 23, returns 15, permanent 8, endorsement 86, intention 76) are unchanged. Band percentages (retention 85.4, commitment gap 29.3 pp) are computed on the rebuilt denominators.</t>
+          <t>Note: all targets follow the participant register (38 / 41 / 41; total 120). An earlier internal draft summary carried 35 / 40 / 45 — superseded; the Paper 3 manuscript is unpublished. Outcome-count targets (dropouts 23, returns 15, permanent 8, endorsement 86, intention 76) unchanged. Band percentages (retention 85.4, commitment gap 29.3 pp) computed on the register denominators.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage-3: archive second data file as self-declared synthetic; no merge
The 21/07 'Constrained_Telemetry' file's own Validation sheet states
'Dataset status: Synthetic / constrained simulation' with participant
IDs 'randomly distributed across behavioural groups' - it passes all 26
registered targets because it was generated under them. Archived as a
labelled artifact alongside the 19/07 file (whose content contradicts
it). Analysis sheets remain empty; thesis unchanged, resting on the
preliminary aggregate record.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
+++ b/docs/thesis/Stage3_Data_Logbook_120cases_with_Reconciliation.xlsx
@@ -23509,6 +23509,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>UPDATE 25 Jul 2026: a second file received the same week ('...Registered_Results_Constrained_Telemetry.xlsx') declares itself in its own Validation sheet as 'Synthetic / constrained simulation' built to pass the registered targets, and its participant-level content contradicts this sheet's content. Neither file can serve as the transcribed participant-level record. Both are archived under data_entry/ as labelled artifacts. The analysis sheets remain empty pending transcription from genuine primary records.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>